<commit_message>
Lagerplatzänderung vereinfachen, Mitarbeiter ergänzen, SAP-Exportformat für Massenkorrektur
- "Bisheriger Lagerplatz" aus Lagerplatzänderung entfernt (Formular, Excel-
  Export, Startseiten-Anzeige) - wird nicht benötigt, nur noch der neue
  Lagerplatz wird erfasst.
- "Esser, Markus" zur Mitarbeiterliste (data/mitarbeiter.xlsx) ergänzt.
- Massen-Lagerplatzkorrektur exportiert jetzt im festen SAP-Massenupload-
  Format (siehe "Lageraort Massen - Ausgabeliste.xlsx"): Spalten MATNR
  (Artikelnummer), WERKS/LGORT (fest "106"), LGPBE (neuer Lagerplatz) -
  keine weiteren Spalten mehr, damit die Datei direkt in den SAP-Upload
  passt.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/mitarbeiter.xlsx
+++ b/data/mitarbeiter.xlsx
@@ -1,82 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sigplc-my.sharepoint.com/personal/markus_esser_wego-vti_de/Documents/Desktop/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_9A265F44C4094E7AB8558C05BD940E073B8A9C6D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B3DB81E-2B7D-4FB0-B4AA-621B95B609AD}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="1188" windowWidth="34560" windowHeight="24732" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5760" yWindow="1188" windowWidth="34560" windowHeight="24732" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
-  <si>
-    <t>Berisha, Selim</t>
-  </si>
-  <si>
-    <t>Blensekemper, Marcel</t>
-  </si>
-  <si>
-    <t>Büchner, Sören</t>
-  </si>
-  <si>
-    <t>Giermann, Levin</t>
-  </si>
-  <si>
-    <t>Hein, Viktor</t>
-  </si>
-  <si>
-    <t>Hein, Marco</t>
-  </si>
-  <si>
-    <t>Jochheim, Martin</t>
-  </si>
-  <si>
-    <t>Liermann, Rene</t>
-  </si>
-  <si>
-    <t>Klaes, Marcel</t>
-  </si>
-  <si>
-    <t>Obermeyer, Ralf</t>
-  </si>
-  <si>
-    <t>Surmann, Steffen</t>
-  </si>
-  <si>
-    <t>Schlamann, Thomas</t>
-  </si>
-  <si>
-    <t>Wels, Mark</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <name val="Arial"/>
       <sz val="10"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -115,29 +63,89 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{D16222E5-51C9-41DA-AE62-0BAB1F03A49F}"/>
+    <tableStyle name="Invisible" pivot="0" table="0" count="0"/>
   </tableStyles>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -457,92 +465,123 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col width="22" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>12</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>Berisha, Selim</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>Blensekemper, Marcel</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>Büchner, Sören</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>Giermann, Levin</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Hein, Viktor</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Hein, Marco</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>Jochheim, Martin</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Liermann, Rene</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Klaes, Marcel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Obermeyer, Ralf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>Surmann, Steffen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>Schlamann, Thomas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>Wels, Mark</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Esser, Markus</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter alignWithMargins="0"/>
 </worksheet>
-</file>
-
-<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
-<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{636bb9a7-f223-444d-9af6-d85e7a533374}" enabled="0" method="" siteId="{636bb9a7-f223-444d-9af6-d85e7a533374}" removed="1"/>
-</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
15 neue Mitarbeiter zur Mitarbeiterliste (Standort 106) hinzugefügt
Teigelkamp/Ralf, Schulte/Linda, Holberndt/Hendrik, Krumme/Stephan,
Büker/Christian, Hövel/Felix, Schürmann/Felix, Völkoi/Tobias, Krause/Andre,
Beilmann/Ralf, Kuhlage/Jürgen, Schwering/Stefan, Ratermann/Sven,
Reshetnik/Maxim, Brockel/Linus.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/mitarbeiter.xlsx
+++ b/data/mitarbeiter.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="13.2"/>
   <cols>
     <col width="22" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -575,9 +575,114 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>Esser, Markus</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>Teigelkamp, Ralf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>Schulte, Linda</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>Holberndt, Hendrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>Krumme, Stephan</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>Büker, Christian</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>Hövel, Felix</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>Schürmann, Felix</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Völkoi, Tobias</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>Krause, Andre</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>Beilmann, Ralf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t>Kuhlage, Jürgen</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>Schwering, Stefan</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>Ratermann, Sven</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>Reshetnik, Maxim</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>Brockel, Linus</t>
         </is>
       </c>
     </row>

</xml_diff>